<commit_message>
Exp3 EDA checkpoint: readable labels + reward-hacking figures (pre-reorg)
Snapshot before the reorg-by-topic pass. Includes: central DISPLAY_NAMES/
arm_label label layer, reward_hack_panel, mark_peaks trajectory annotation,
orthogonal effect forest + lower_is_better, heterogeneity refinements +
subgroup_endpoint_bars, question_rate_crosscheck, L2 view staging
(config/render_views/oracle_scoring), regenerated L0 view.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Exp3_PTO_GRPO/eda/results/L0/tables/eval/eval.xlsx
+++ b/Exp3_PTO_GRPO/eda/results/L0/tables/eval/eval.xlsx
@@ -431,59 +431,59 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Q1Q2</t>
+          <t>Satisfaction (Q1+Q2)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>WAI-SR</t>
+          <t>Working Alliance</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>CSQ-8</t>
+          <t>Client Satisfaction</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>MI-SAT</t>
+          <t>MI Satisfaction</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>MITI</t>
+          <t>MI Integrity</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>PCT</t>
+          <t>Patient Change-Talk</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>MICI ↓</t>
+          <t>MI-Inconsistency ↓</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>R:Q</t>
+          <t>Reflection:Question</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>%CR</t>
+          <t>% Complex Reflections</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>%MICO</t>
+          <t>% MI-Consistent</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PTO_LA0</t>
+          <t>PTO (K=0)</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -523,7 +523,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GRPO_LA0</t>
+          <t>GRPO (K=0)</t>
         </is>
       </c>
       <c r="B3" t="n">

</xml_diff>